<commit_message>
Add sales KPI analysis Excel practice
</commit_message>
<xml_diff>
--- a/day3_excel_practise.xlsx
+++ b/day3_excel_practise.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZUNAIRA\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C109B12-B0E0-495A-91C7-B04ECE8035BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545D1FFF-AB51-4775-A99B-6CC37B42C38D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{0B42CB26-DCA2-41DE-B6F4-906051939585}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{0B42CB26-DCA2-41DE-B6F4-906051939585}"/>
   </bookViews>
   <sheets>
     <sheet name="data cleaning" sheetId="1" r:id="rId1"/>
+    <sheet name="KPI SHEET" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
   <si>
     <t>Employee ID</t>
   </si>
@@ -100,13 +101,127 @@
   </si>
   <si>
     <t>Department Result</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Latte</t>
+  </si>
+  <si>
+    <t>Cappuccino</t>
+  </si>
+  <si>
+    <t>Tea</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Coffee</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Revenue.</t>
+  </si>
+  <si>
+    <t>KPI</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>TOTAL REVENUE</t>
+  </si>
+  <si>
+    <t>TEA REVENUE</t>
+  </si>
+  <si>
+    <t>Total Sales Revenue</t>
+  </si>
+  <si>
+    <r>
+      <t>Coffee Sales Count</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Tea Sales Count</t>
+  </si>
+  <si>
+    <t>Average Sale Value</t>
+  </si>
+  <si>
+    <t>Coffee Revenue %</t>
+  </si>
+  <si>
+    <t>MoM Growth (Feb 2025)</t>
+  </si>
+  <si>
+    <r>
+      <t>YoY Growth (Jan)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Month.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SALES KPI ANALYSIS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,16 +229,58 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -131,11 +288,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -145,9 +321,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="5">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Good" xfId="3" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -460,7 +661,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{180B6D19-C272-435D-AC23-F983CF07A400}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.85546875" customWidth="1"/>
     <col min="2" max="2" width="23.140625" customWidth="1"/>
@@ -471,7 +672,7 @@
     <col min="8" max="8" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -495,7 +696,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -522,7 +723,7 @@
         <v>IT</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -544,7 +745,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -566,7 +767,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -588,7 +789,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -614,4 +815,305 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D64E3DBA-0EBA-4657-ADF4-65DB130D8D16}">
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="5.5703125" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="6">
+        <v>45662</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="8">
+        <v>10</v>
+      </c>
+      <c r="E2" s="8">
+        <v>150</v>
+      </c>
+      <c r="F2" s="9">
+        <f>D2*E2</f>
+        <v>1500</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="11">
+        <f>SUMIFS(F2:F7,C2:C7,"Coffee")</f>
+        <v>6840</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="6">
+        <v>45669</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="8">
+        <v>8</v>
+      </c>
+      <c r="E3" s="8">
+        <v>180</v>
+      </c>
+      <c r="F3" s="9">
+        <f t="shared" ref="F3:F7" si="0">D3*E3</f>
+        <v>1440</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="11">
+        <f>SUMIFS(F2:F7,C2:C7,"Tea")</f>
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="6">
+        <v>45691</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="8">
+        <v>12</v>
+      </c>
+      <c r="E4" s="8">
+        <v>150</v>
+      </c>
+      <c r="F4" s="9">
+        <f t="shared" si="0"/>
+        <v>1800</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="11">
+        <f>SUM(F2:F7)</f>
+        <v>10340</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="6">
+        <v>45702</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="8">
+        <v>15</v>
+      </c>
+      <c r="E5" s="8">
+        <v>100</v>
+      </c>
+      <c r="F5" s="9">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" s="11">
+        <f>COUNTIFS(C2:C7,"Coffee")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="6">
+        <v>46030</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="8">
+        <v>14</v>
+      </c>
+      <c r="E6" s="8">
+        <v>150</v>
+      </c>
+      <c r="F6" s="9">
+        <f t="shared" si="0"/>
+        <v>2100</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" s="11">
+        <f>COUNTIFS(C2:C7,"TEA")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="6">
+        <v>46063</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="8">
+        <v>20</v>
+      </c>
+      <c r="E7" s="8">
+        <v>100</v>
+      </c>
+      <c r="F7" s="9">
+        <f t="shared" si="0"/>
+        <v>2000</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="11">
+        <f>AVERAGE(F2:F7)</f>
+        <v>1723.3333333333333</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="H8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="13">
+        <f>I2/I4</f>
+        <v>0.66150870406189555</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="18">
+      <c r="A9" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="H10" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="H11" s="14">
+        <v>45658</v>
+      </c>
+      <c r="I11" s="11">
+        <f>SUMIFS(F2:F7,A2:A7,"&gt;=2025-01-01",A2:A7,"&lt;=2025-01-31")</f>
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="H12" s="14">
+        <v>45689</v>
+      </c>
+      <c r="I12" s="11">
+        <f>SUMIFS(F2:F7,A2:A7,"&gt;=2025-02-01",A2:A7,"&lt;=2025-02-28")</f>
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="H13" s="14">
+        <v>46023</v>
+      </c>
+      <c r="I13" s="11">
+        <f>SUMIFS(F2:F7,A2:A7,"&gt;=2026-01-01",A2:A7,"&lt;=2026-01-31")</f>
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="H14" s="14">
+        <v>46054</v>
+      </c>
+      <c r="I14" s="11">
+        <f>SUMIFS(F2:F7,A2:A7,"&gt;=2026-02-01",A2:A7,"&lt;=2026-02-28")</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="H15" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I15" s="7">
+        <f>(I12-I11)/I11</f>
+        <v>0.12244897959183673</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="H16" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="I16" s="13">
+        <f>(I13-I11)/I11</f>
+        <v>-0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="19" spans="6:6">
+      <c r="F19" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A9:F9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>